<commit_message>
NACIE TECDOC: add IGCAR v01 source files
</commit_message>
<xml_diff>
--- a/01-source/annex-II-organizations/ALL_PARTICIPANTS.xlsx
+++ b/01-source/annex-II-organizations/ALL_PARTICIPANTS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikityuk\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikityuk\AppData\Local\Temp\_tc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD21D176-1FD0-4FF4-A8BA-BA188648AD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC78574-827A-4546-A026-06E9DB4E54D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{403AE6FC-82DD-4955-9E6C-08160414FA22}"/>
   </bookViews>
@@ -793,12 +793,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -813,9 +819,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1422,25 +1429,29 @@
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F13" t="s">
-        <v>16</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="E13" s="2"/>
+      <c r="F13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K13" t="s">
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>